<commit_message>
Pour la Recupération de la version nouvelle
</commit_message>
<xml_diff>
--- a/media/uploaded_files/Test1.xlsx
+++ b/media/uploaded_files/Test1.xlsx
@@ -9,11 +9,13 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7500" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7500" activeTab="3"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
-    <sheet name="Feuil2" sheetId="2" r:id="rId2"/>
+    <sheet name="EII1" sheetId="1" r:id="rId1"/>
+    <sheet name="RT2" sheetId="3" r:id="rId2"/>
+    <sheet name="EII3" sheetId="4" r:id="rId3"/>
+    <sheet name="BTP2" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="43">
   <si>
     <t>HEURES</t>
   </si>
@@ -982,9 +984,681 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:7" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="10"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="12"/>
+    </row>
+    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="G8" s="13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G9" s="13" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="G10" s="20" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:7" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="10"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="12"/>
+    </row>
+    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="G8" s="13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G9" s="13" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="G10" s="20" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="C1:I11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="3:9" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="C1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="3:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="C2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="3:9" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="C3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C6" s="10"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="12"/>
+    </row>
+    <row r="7" spans="3:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="C7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="3:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="C8" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I8" s="13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C9" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H9" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="I9" s="13" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="3:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C10" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="G10" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="H10" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="I10" s="20" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="3:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>